<commit_message>
chore(research): regenerar los visuales de la encuesta con paleta validada
Los graficos pasan a la serie categorica "Pulso Vital", validada
todos-contra-todos, y a una rampa ordinal de un solo tono (laton) monotona
en luminancia, que sigue siendo legible en escala de grises y para quien
no distingue los hues.

Se anade generar_visuales.py, el script que los produce, y se elimina el
dashboard_ondigital(1).html duplicado.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011g9zaZFmJibnnX4TSPsZAo
</commit_message>
<xml_diff>
--- a/ONDIGITAL_Analisis_Encuesta/ONDIGITAL_Analisis_Completo.xlsx
+++ b/ONDIGITAL_Analisis_Encuesta/ONDIGITAL_Analisis_Completo.xlsx
@@ -28,9 +28,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -41,59 +42,59 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Aptos Display"/>
+      <name val="Fraunces"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="24"/>
     </font>
     <font>
-      <name val="Aptos"/>
+      <name val="Inter"/>
       <i val="1"/>
-      <color rgb="005D6D81"/>
+      <color rgb="005F5B4E"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="003B82F6"/>
+      <color rgb="008C6A2A"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Aptos Display"/>
+      <name val="Fraunces"/>
       <b val="1"/>
-      <color rgb="000B1A2E"/>
+      <color rgb="000B1410"/>
       <sz val="22"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="005D6D81"/>
+      <color rgb="005F5B4E"/>
     </font>
     <font>
-      <color rgb="000B1A2E"/>
+      <color rgb="000B1410"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="003B82F6"/>
+      <color rgb="008C6A2A"/>
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="000B1A2E"/>
+      <color rgb="000B1410"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="008A5A00"/>
+      <color rgb="006E5320"/>
       <sz val="12"/>
     </font>
     <font>
-      <color rgb="006D4A00"/>
+      <color rgb="005A4419"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="003B82F6"/>
+      <color rgb="008C6A2A"/>
     </font>
     <font>
-      <color rgb="005D6D81"/>
+      <color rgb="005F5B4E"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -104,43 +105,43 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B1A2E"/>
+      <color rgb="000B1410"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Aptos"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Aptos"/>
-      <color rgb="000B1A2E"/>
+      <name val="Inter"/>
+      <color rgb="000B1410"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="005D6D81"/>
+      <color rgb="005F5B4E"/>
       <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B1A2E"/>
+      <color rgb="000B1410"/>
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="000B1A2E"/>
+      <color rgb="000B1410"/>
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="006D4A00"/>
+      <color rgb="005A4419"/>
     </font>
     <font>
-      <color rgb="005D6D81"/>
+      <color rgb="005F5B4E"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B1A2E"/>
+      <color rgb="000B1410"/>
     </font>
   </fonts>
   <fills count="8">
@@ -152,32 +153,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00071426"/>
+        <fgColor rgb="000B1410"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF3FF"/>
+        <fgColor rgb="00F7EEDC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6FBF5"/>
+        <fgColor rgb="00E4F3EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF5DD"/>
+        <fgColor rgb="00FBF0D8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7FAFD"/>
+        <fgColor rgb="00FAF8F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003B82F6"/>
+        <fgColor rgb="008C6A2A"/>
       </patternFill>
     </fill>
   </fills>
@@ -191,91 +192,91 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B9D5F7"/>
+        <color rgb="00D9C49B"/>
       </left>
       <right style="thin">
-        <color rgb="00B9D5F7"/>
+        <color rgb="00D9C49B"/>
       </right>
       <top style="thin">
-        <color rgb="00B9D5F7"/>
+        <color rgb="00D9C49B"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B9D5F7"/>
+        <color rgb="00D9C49B"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D5DFEB"/>
+        <color rgb="00DBD5C4"/>
       </left>
       <right style="thin">
-        <color rgb="00D5DFEB"/>
+        <color rgb="00DBD5C4"/>
       </right>
       <top style="thin">
-        <color rgb="00D5DFEB"/>
+        <color rgb="00DBD5C4"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D5DFEB"/>
+        <color rgb="00DBD5C4"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B7E8DA"/>
+        <color rgb="00B4D9C7"/>
       </left>
       <right style="thin">
-        <color rgb="00B7E8DA"/>
+        <color rgb="00B4D9C7"/>
       </right>
       <top style="thin">
-        <color rgb="00B7E8DA"/>
+        <color rgb="00B4D9C7"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B7E8DA"/>
+        <color rgb="00B4D9C7"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00F1D38A"/>
+        <color rgb="00E8CE95"/>
       </left>
       <right style="thin">
-        <color rgb="00F1D38A"/>
+        <color rgb="00E8CE95"/>
       </right>
       <top style="thin">
-        <color rgb="00F1D38A"/>
+        <color rgb="00E8CE95"/>
       </top>
       <bottom style="thin">
-        <color rgb="00F1D38A"/>
+        <color rgb="00E8CE95"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00071426"/>
+        <color rgb="000B1410"/>
       </left>
       <right style="thin">
-        <color rgb="00071426"/>
+        <color rgb="000B1410"/>
       </right>
       <top style="thin">
-        <color rgb="00071426"/>
+        <color rgb="000B1410"/>
       </top>
       <bottom style="thin">
-        <color rgb="00071426"/>
+        <color rgb="000B1410"/>
       </bottom>
     </border>
     <border>
       <bottom style="hair">
-        <color rgb="00D5DFEB"/>
+        <color rgb="00DBD5C4"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="003B82F6"/>
+        <color rgb="008C6A2A"/>
       </left>
       <right style="thin">
-        <color rgb="003B82F6"/>
+        <color rgb="008C6A2A"/>
       </right>
       <top style="thin">
-        <color rgb="003B82F6"/>
+        <color rgb="008C6A2A"/>
       </top>
       <bottom style="thin">
-        <color rgb="003B82F6"/>
+        <color rgb="008C6A2A"/>
       </bottom>
     </border>
   </borders>
@@ -283,7 +284,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -353,11 +354,18 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="16" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -367,14 +375,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00E6FBF5"/>
+          <fgColor rgb="00E4F3EC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFE9EC"/>
+          <fgColor rgb="00FBE4E1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -683,7 +691,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4953000" cy="3000375"/>
+    <ext cx="4953000" cy="1971675"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -708,7 +716,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4953000" cy="3000375"/>
+    <ext cx="4953000" cy="1971675"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -733,7 +741,7 @@
       <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4953000" cy="2705100"/>
+    <ext cx="4953000" cy="2247900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -758,7 +766,7 @@
       <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4953000" cy="3000375"/>
+    <ext cx="4953000" cy="1971675"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -868,19 +876,22 @@
     <tableColumn id="1" name="Bloque"/>
     <tableColumn id="2" name="Respuesta/Categoria"/>
     <tableColumn id="3" name="Frecuencia"/>
-    <tableColumn id="4" name="Porcentaje"/>
+    <tableColumn id="4" name="Porcentaje (% de 321 respuestas)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TblAsociaciones" displayName="TblAsociaciones" ref="A6:C17" headerRowCount="1">
-  <autoFilter ref="A6:C17"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TblAsociaciones" displayName="TblAsociaciones" ref="A6:F17" headerRowCount="1">
+  <autoFilter ref="A6:F17"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="Relacion"/>
-    <tableColumn id="2" name="Efecto (V o rho)"/>
-    <tableColumn id="3" name="p_value"/>
+    <tableColumn id="2" name="Prueba"/>
+    <tableColumn id="3" name="Efecto"/>
+    <tableColumn id="4" name="p_value"/>
+    <tableColumn id="5" name="n"/>
+    <tableColumn id="6" name="Nota"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1185,7 +1196,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0000E5B0"/>
+    <tabColor rgb="00D8A24A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1212,7 +1223,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Paquete ejecutivo de análisis de encuesta · generado el 2026-08-16</t>
+          <t>Paquete ejecutivo de análisis de encuesta · generado el 2026-09-02</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1491,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="003B82F6"/>
+    <tabColor rgb="008C6A2A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1629,7 +1640,7 @@
       <c r="D9" s="19" t="n"/>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
       <c r="F9" s="19" t="n">
@@ -1917,7 +1928,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0000E5B0"/>
+    <tabColor rgb="00D8A24A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2210,7 +2221,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="007FA7D8"/>
+    <tabColor rgb="006C35ED"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -12047,7 +12058,7 @@
       </c>
       <c r="X97" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -12151,7 +12162,7 @@
       </c>
       <c r="X98" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -12567,7 +12578,7 @@
       </c>
       <c r="X102" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12786,7 @@
       </c>
       <c r="X104" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -13295,7 +13306,7 @@
       </c>
       <c r="X109" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -13607,7 +13618,7 @@
       </c>
       <c r="X112" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -14127,7 +14138,7 @@
       </c>
       <c r="X117" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -14647,7 +14658,7 @@
       </c>
       <c r="X122" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -14855,7 +14866,7 @@
       </c>
       <c r="X124" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -15271,7 +15282,7 @@
       </c>
       <c r="X128" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -15375,7 +15386,7 @@
       </c>
       <c r="X129" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -15583,7 +15594,7 @@
       </c>
       <c r="X131" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -15791,7 +15802,7 @@
       </c>
       <c r="X133" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -15895,7 +15906,7 @@
       </c>
       <c r="X134" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -16415,7 +16426,7 @@
       </c>
       <c r="X139" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -16519,7 +16530,7 @@
       </c>
       <c r="X140" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -16623,7 +16634,7 @@
       </c>
       <c r="X141" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -16831,7 +16842,7 @@
       </c>
       <c r="X143" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -17247,7 +17258,7 @@
       </c>
       <c r="X147" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -17663,7 +17674,7 @@
       </c>
       <c r="X151" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -17975,7 +17986,7 @@
       </c>
       <c r="X154" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -18183,7 +18194,7 @@
       </c>
       <c r="X156" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -18807,7 +18818,7 @@
       </c>
       <c r="X162" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -19015,7 +19026,7 @@
       </c>
       <c r="X164" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -19223,7 +19234,7 @@
       </c>
       <c r="X166" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -19327,7 +19338,7 @@
       </c>
       <c r="X167" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -20055,7 +20066,7 @@
       </c>
       <c r="X174" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -20263,7 +20274,7 @@
       </c>
       <c r="X176" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -20887,7 +20898,7 @@
       </c>
       <c r="X182" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -20991,7 +21002,7 @@
       </c>
       <c r="X183" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -21095,7 +21106,7 @@
       </c>
       <c r="X184" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -21199,7 +21210,7 @@
       </c>
       <c r="X185" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -21407,7 +21418,7 @@
       </c>
       <c r="X187" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -21511,7 +21522,7 @@
       </c>
       <c r="X188" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -21615,7 +21626,7 @@
       </c>
       <c r="X189" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -22135,7 +22146,7 @@
       </c>
       <c r="X194" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -22343,7 +22354,7 @@
       </c>
       <c r="X196" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -23071,7 +23082,7 @@
       </c>
       <c r="X203" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -23279,7 +23290,7 @@
       </c>
       <c r="X205" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -23695,7 +23706,7 @@
       </c>
       <c r="X209" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -24007,7 +24018,7 @@
       </c>
       <c r="X212" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -24215,7 +24226,7 @@
       </c>
       <c r="X214" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -24631,7 +24642,7 @@
       </c>
       <c r="X218" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -25255,7 +25266,7 @@
       </c>
       <c r="X224" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -25359,7 +25370,7 @@
       </c>
       <c r="X225" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -25671,7 +25682,7 @@
       </c>
       <c r="X228" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -25775,7 +25786,7 @@
       </c>
       <c r="X229" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -25879,7 +25890,7 @@
       </c>
       <c r="X230" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -25983,7 +25994,7 @@
       </c>
       <c r="X231" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -26087,7 +26098,7 @@
       </c>
       <c r="X232" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -26399,7 +26410,7 @@
       </c>
       <c r="X235" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -26503,7 +26514,7 @@
       </c>
       <c r="X236" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26618,7 @@
       </c>
       <c r="X237" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -26919,7 +26930,7 @@
       </c>
       <c r="X240" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -27023,7 +27034,7 @@
       </c>
       <c r="X241" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -27231,7 +27242,7 @@
       </c>
       <c r="X243" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -27647,7 +27658,7 @@
       </c>
       <c r="X247" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -27959,7 +27970,7 @@
       </c>
       <c r="X250" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -28479,7 +28490,7 @@
       </c>
       <c r="X255" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -28687,7 +28698,7 @@
       </c>
       <c r="X257" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -28895,7 +28906,7 @@
       </c>
       <c r="X259" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -29103,7 +29114,7 @@
       </c>
       <c r="X261" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -29311,7 +29322,7 @@
       </c>
       <c r="X263" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29426,7 @@
       </c>
       <c r="X264" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -29727,7 +29738,7 @@
       </c>
       <c r="X267" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -30039,7 +30050,7 @@
       </c>
       <c r="X270" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -30143,7 +30154,7 @@
       </c>
       <c r="X271" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -30455,7 +30466,7 @@
       </c>
       <c r="X274" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -30767,7 +30778,7 @@
       </c>
       <c r="X277" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -30871,7 +30882,7 @@
       </c>
       <c r="X278" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -30975,7 +30986,7 @@
       </c>
       <c r="X279" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -31183,7 +31194,7 @@
       </c>
       <c r="X281" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -31599,7 +31610,7 @@
       </c>
       <c r="X285" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -31703,7 +31714,7 @@
       </c>
       <c r="X286" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -31807,7 +31818,7 @@
       </c>
       <c r="X287" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -32327,7 +32338,7 @@
       </c>
       <c r="X292" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -33055,7 +33066,7 @@
       </c>
       <c r="X299" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -33679,7 +33690,7 @@
       </c>
       <c r="X305" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -33887,7 +33898,7 @@
       </c>
       <c r="X307" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -33991,7 +34002,7 @@
       </c>
       <c r="X308" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -34303,7 +34314,7 @@
       </c>
       <c r="X311" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -34615,7 +34626,7 @@
       </c>
       <c r="X314" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -34823,7 +34834,7 @@
       </c>
       <c r="X316" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -35031,7 +35042,7 @@
       </c>
       <c r="X318" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -35447,7 +35458,7 @@
       </c>
       <c r="X322" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -35551,7 +35562,7 @@
       </c>
       <c r="X323" s="19" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -35655,7 +35666,7 @@
       </c>
       <c r="X324" s="15" t="inlineStr">
         <is>
-          <t>Interes medio / diagnostico</t>
+          <t>Interés medio / diagnóstico</t>
         </is>
       </c>
     </row>
@@ -35775,9 +35786,9 @@
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="00FF6B75"/>
-        <color rgb="00F9B84A"/>
-        <color rgb="0049D18E"/>
+        <color rgb="00E85D4E"/>
+        <color rgb="00E0A83D"/>
+        <color rgb="002FA277"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -35800,7 +35811,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00F9B84A"/>
+    <tabColor rgb="00E0A83D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -35849,7 +35860,7 @@
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Porcentaje</t>
+          <t>Porcentaje (% de 321 respuestas)</t>
         </is>
       </c>
       <c r="E4" s="14" t="n"/>
@@ -36036,7 +36047,7 @@
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q3 (combinaciones exclusivas)</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
@@ -36058,7 +36069,7 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q3 (combinaciones exclusivas)</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -36080,7 +36091,7 @@
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q3 (combinaciones exclusivas)</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
@@ -36102,7 +36113,7 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q3 (combinaciones exclusivas)</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
@@ -36124,7 +36135,7 @@
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q3 (combinaciones exclusivas)</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
@@ -36146,7 +36157,7 @@
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q3 (combinaciones exclusivas)</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -36168,7 +36179,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q3 (combinaciones exclusivas)</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -36652,7 +36663,7 @@
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>Q9 (multiseleccion)</t>
+          <t>Q9 (multiseleccion sobre 321 personas)</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -36674,7 +36685,7 @@
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>Q9 (multiseleccion)</t>
+          <t>Q9 (multiseleccion sobre 321 personas)</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
@@ -36696,7 +36707,7 @@
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>Q9 (multiseleccion)</t>
+          <t>Q9 (multiseleccion sobre 321 personas)</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -36718,7 +36729,7 @@
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>Q9 (multiseleccion)</t>
+          <t>Q9 (multiseleccion sobre 321 personas)</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
@@ -37963,23 +37974,26 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00FF6B75"/>
+    <tabColor rgb="00E85D4E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -38002,7 +38016,7 @@
           <t>Asociaciones principales</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Control de calidad</t>
         </is>
@@ -38016,185 +38030,274 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Efecto (V o rho)</t>
+          <t>Prueba</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
+          <t>Efecto</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="27" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="27" t="inlineStr">
         <is>
           <t>Respuestas abiertas con plantilla</t>
         </is>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="I6" s="28" t="n">
         <v>321</v>
       </c>
-      <c r="G6" s="14" t="n"/>
-      <c r="H6" s="14" t="n"/>
-      <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Madurez tecnologica vs disposicion</t>
+          <t>Madurez tecnológica vs disposición</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>0.442</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>2.7413209974729543e-37</t>
-        </is>
-      </c>
-      <c r="E7" s="29" t="inlineStr">
+          <t>V de Cramér corregida (sin signo)</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>0.442</v>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>321</v>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Mide fuerza de asociación, no dirección. Tabla 4x4, todas las frecuencias esperadas &gt;= 9.</t>
+        </is>
+      </c>
+      <c r="H7" s="30" t="inlineStr">
         <is>
           <t>Pares en el mismo segundo</t>
         </is>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="I7" s="31" t="n">
         <v>176</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Tiempo perdido vs disposicion</t>
+          <t>Tiempo perdido vs disposición</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>0.453</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>3.223824434937886e-39</t>
-        </is>
-      </c>
-      <c r="E8" s="29" t="inlineStr">
+          <t>V de Cramér corregida (sin signo)</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>321</v>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>Asociación moderada. Tabla 4x4, frecuencias esperadas &gt;= 11.</t>
+        </is>
+      </c>
+      <c r="H8" s="30" t="inlineStr">
         <is>
           <t>Pares ≤ 2 segundos</t>
         </is>
       </c>
-      <c r="F8" s="30" t="n">
+      <c r="I8" s="31" t="n">
         <v>296</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="46" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Freno principal vs disposicion</t>
+          <t>Freno principal vs disposición</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>0.434</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>7.007242926808732e-36</t>
-        </is>
-      </c>
-      <c r="E9" s="29" t="inlineStr">
+          <t>V de Cramér corregida (sin signo)</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>321</v>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Asociación moderada. Tabla 4x4, frecuencias esperadas &gt;= 9.</t>
+        </is>
+      </c>
+      <c r="H9" s="30" t="inlineStr">
         <is>
           <t>Filas en patrones cerrados</t>
         </is>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="I9" s="31" t="n">
         <v>75</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="46" customHeight="1">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Equipo externo vs disposicion</t>
+          <t>Equipo externo vs disposición</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>0.419</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>2.7209227673381574e-33</t>
-        </is>
-      </c>
-      <c r="E10" s="29" t="inlineStr">
+          <t>V de Cramér corregida (sin signo)</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>321</v>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>Asociación moderada. Tabla 4x4, frecuencias esperadas &gt;= 10.</t>
+        </is>
+      </c>
+      <c r="H10" s="30" t="inlineStr">
         <is>
           <t>Duración de captura (s)</t>
         </is>
       </c>
-      <c r="F10" s="30" t="n">
+      <c r="I10" s="31" t="n">
         <v>1499</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="46" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Aprendizaje vs disposicion</t>
+          <t>Aprendizaje vs disposición</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>0.418</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>4.277273854137304e-33</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
+          <t>V de Cramér corregida (sin signo)</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>321</v>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Asociación moderada. Tabla 4x4, frecuencias esperadas &gt;= 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Almacenamiento vs percepcion de perdida</t>
+          <t>Almacenamiento vs percepción de pérdida</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>0.236</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>2.432552318059986e-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+          <t>V de Cramér corregida (sin signo)</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>no fiable</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>321</v>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>ADVERTENCIA: tabla 7x5 con 20 de 35 celdas de frecuencia esperada &lt; 5 (mínimo 0.45). La aproximación chi-cuadrado no se sostiene; tomar solo como indicio y reagrupar categorías antes de citarla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Madurez vs disposicion (Spearman)</t>
+          <t>Madurez vs disposición (Spearman)</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>-0.201</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
-        <is>
-          <t>0.00029570583263715405</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Lectura</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+          <t>rho de Spearman (con signo)</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>-0.201</v>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>321</v>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Negativa: a mayor madurez declarada, menor disposición. No contradice la fila 1: la V mide asociación total y esta rho mide solo la tendencia monótona.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Cómo leer esta tabla</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Horas perdidas vs dolor (Spearman)</t>
@@ -38202,55 +38305,88 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>0.177</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>0.0014139575970666387</t>
-        </is>
-      </c>
-      <c r="E14" s="31" t="inlineStr">
-        <is>
-          <t>La asociación más fuerte del archivo es equipo externo vs aprendizaje (rho = 0.638). También aparecen relaciones moderadas entre tiempo perdido, madurez, frenos y disposición. Úsalas para priorizar preguntas de validación, no como evidencia causal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
+          <t>rho de Spearman (con signo)</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>321</v>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>Efecto pequeño; sirve como hipótesis a validar en entrevistas.</t>
+        </is>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>Todas las filas se calculan sobre las mismas n = 321 respuestas. La V de Cramér (corregida por sesgo) mide fuerza de asociación entre variables nominales y nunca es negativa; la rho de Spearman mide la tendencia monótona y sí lleva signo, por eso madurez vs disposición aparece dos veces con valores distintos y no es una contradicción. La asociación más fuerte del archivo es equipo externo vs aprendizaje (rho = 0.638). La fila de almacenamiento vs percepción de pérdida no cumple el supuesto de chi-cuadrado (20 de 35 celdas con frecuencia esperada &lt; 5): no citarla como resultado significativo. Nada de esto prueba causalidad ni representatividad del mercado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>Disposicion vs equipo externo (Spearman)</t>
+          <t>Disposición vs equipo externo (Spearman)</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>0.144</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>0.00959895555569453</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
+          <t>rho de Spearman (con signo)</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>0.010</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>321</v>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Efecto pequeño; el más débil del archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Disposicion vs aprendizaje (Spearman)</t>
+          <t>Disposición vs aprendizaje (Spearman)</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>0.218</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>8.253256188566585e-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+          <t>rho de Spearman (con signo)</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="n">
+        <v>0.218</v>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>321</v>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Efecto pequeño a moderado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>Equipo externo vs aprendizaje (Spearman)</t>
@@ -38258,31 +38394,44 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0.638</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>4.1617810216990873e-38</t>
+          <t>rho de Spearman (con signo)</t>
+        </is>
+      </c>
+      <c r="C17" s="34" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>&lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>321</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Asociación más fuerte del archivo; coherente con el argumento comercial del plan Business.</t>
         </is>
       </c>
     </row>
     <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="E14:J18"/>
+    <mergeCell ref="H14:M20"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:B17">
+  <conditionalFormatting sqref="C7:C17">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="00FFE9EC"/>
-        <color rgb="00FFF5DD"/>
-        <color rgb="00E6FBF5"/>
+        <color rgb="00FBE4E1"/>
+        <color rgb="00FBF0D8"/>
+        <color rgb="00E4F3EC"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -38297,7 +38446,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00F9B84A"/>
+    <tabColor rgb="00E0A83D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -38634,7 +38783,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="007FA7D8"/>
+    <tabColor rgb="006C35ED"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>